<commit_message>
Cards: fix audience_score for the 37 new films — use Metacritic USER score, not the critics Metascore
The "Metacritic User Rating" column feeds the audience-score blend with
the Metacritic *user* score ×10 (verified against 11 existing rows:
Dark Knight 9.1→91, Parasite 8.8→88, Joker 8.9→89, …). The initial
import scraped the ld+json ratingValue, which is the *critics* Metascore.
Re-scraped the user scores (Shang-Chi and GotG Vol. 3 read off the
user-reviews page — the redesigned summary widget shows "TBD"). Biggest
moves: Black Panther 81→69, Deadpool & Wolverine 63→74, The Hobbit: An
Unexpected Journey 65→76, Captain Marvel 58→46.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -10649,7 +10649,7 @@
         <v>3.81</v>
       </c>
       <c r="F183" s="10" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H183" s="10">
         <f>ROUND((E183/5*100+F183)/2,0)</f>
@@ -10704,7 +10704,7 @@
         <v>2.58</v>
       </c>
       <c r="F184" s="10" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="H184" s="10">
         <f>ROUND((E184/5*100+F184)/2,0)</f>
@@ -10759,7 +10759,7 @@
         <v>3.07</v>
       </c>
       <c r="F185" s="10" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="H185" s="10">
         <f>ROUND((E185/5*100+F185)/2,0)</f>
@@ -10814,7 +10814,7 @@
         <v>2.89</v>
       </c>
       <c r="F186" s="10" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="H186" s="10">
         <f>ROUND((E186/5*100+F186)/2,0)</f>
@@ -10869,7 +10869,7 @@
         <v>3.38</v>
       </c>
       <c r="F187" s="10" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H187" s="10">
         <f>ROUND((E187/5*100+F187)/2,0)</f>
@@ -10924,7 +10924,7 @@
         <v>3.77</v>
       </c>
       <c r="F188" s="10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H188" s="10">
         <f>ROUND((E188/5*100+F188)/2,0)</f>
@@ -10979,7 +10979,7 @@
         <v>3.14</v>
       </c>
       <c r="F189" s="10" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H189" s="10">
         <f>ROUND((E189/5*100+F189)/2,0)</f>
@@ -11034,7 +11034,7 @@
         <v>2.33</v>
       </c>
       <c r="F190" s="10" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="H190" s="10">
         <f>ROUND((E190/5*100+F190)/2,0)</f>
@@ -11089,7 +11089,7 @@
         <v>3.79</v>
       </c>
       <c r="F191" s="10" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="H191" s="10">
         <f>ROUND((E191/5*100+F191)/2,0)</f>
@@ -11144,7 +11144,7 @@
         <v>3.32</v>
       </c>
       <c r="F192" s="10" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H192" s="10">
         <f>ROUND((E192/5*100+F192)/2,0)</f>
@@ -11199,7 +11199,7 @@
         <v>3.22</v>
       </c>
       <c r="F193" s="10" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="H193" s="10">
         <f>ROUND((E193/5*100+F193)/2,0)</f>
@@ -11254,7 +11254,7 @@
         <v>3.7</v>
       </c>
       <c r="F194" s="10" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H194" s="10">
         <f>ROUND((E194/5*100+F194)/2,0)</f>
@@ -11309,7 +11309,7 @@
         <v>3.5</v>
       </c>
       <c r="F195" s="10" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H195" s="10">
         <f>ROUND((E195/5*100+F195)/2,0)</f>
@@ -11364,7 +11364,7 @@
         <v>3.62</v>
       </c>
       <c r="F196" s="10" t="n">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="H196" s="10">
         <f>ROUND((E196/5*100+F196)/2,0)</f>
@@ -11419,7 +11419,7 @@
         <v>3.51</v>
       </c>
       <c r="F197" s="10" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H197" s="10">
         <f>ROUND((E197/5*100+F197)/2,0)</f>
@@ -11474,7 +11474,7 @@
         <v>3.71</v>
       </c>
       <c r="F198" s="10" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H198" s="10">
         <f>ROUND((E198/5*100+F198)/2,0)</f>
@@ -11529,7 +11529,7 @@
         <v>3.72</v>
       </c>
       <c r="F199" s="10" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="H199" s="10">
         <f>ROUND((E199/5*100+F199)/2,0)</f>
@@ -11584,7 +11584,7 @@
         <v>2.82</v>
       </c>
       <c r="F200" s="10" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H200" s="10">
         <f>ROUND((E200/5*100+F200)/2,0)</f>
@@ -11639,7 +11639,7 @@
         <v>2.63</v>
       </c>
       <c r="F201" s="10" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="H201" s="10">
         <f>ROUND((E201/5*100+F201)/2,0)</f>
@@ -11694,7 +11694,7 @@
         <v>4.02</v>
       </c>
       <c r="F202" s="10" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H202" s="10">
         <f>ROUND((E202/5*100+F202)/2,0)</f>
@@ -11749,7 +11749,7 @@
         <v>3.42</v>
       </c>
       <c r="F203" s="10" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H203" s="10">
         <f>ROUND((E203/5*100+F203)/2,0)</f>
@@ -11804,7 +11804,7 @@
         <v>2.97</v>
       </c>
       <c r="F204" s="10" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H204" s="10">
         <f>ROUND((E204/5*100+F204)/2,0)</f>
@@ -11859,7 +11859,7 @@
         <v>3.4</v>
       </c>
       <c r="F205" s="10" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H205" s="10">
         <f>ROUND((E205/5*100+F205)/2,0)</f>
@@ -11914,7 +11914,7 @@
         <v>2.68</v>
       </c>
       <c r="F206" s="10" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="H206" s="10">
         <f>ROUND((E206/5*100+F206)/2,0)</f>
@@ -12024,7 +12024,7 @@
         <v>2.33</v>
       </c>
       <c r="F208" s="10" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="H208" s="10">
         <f>ROUND((E208/5*100+F208)/2,0)</f>
@@ -12079,7 +12079,7 @@
         <v>3.27</v>
       </c>
       <c r="F209" s="10" t="n">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="H209" s="10">
         <f>ROUND((E209/5*100+F209)/2,0)</f>
@@ -12134,7 +12134,7 @@
         <v>2.14</v>
       </c>
       <c r="F210" s="10" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H210" s="10">
         <f>ROUND((E210/5*100+F210)/2,0)</f>
@@ -12189,7 +12189,7 @@
         <v>3.99</v>
       </c>
       <c r="F211" s="10" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="H211" s="10">
         <f>ROUND((E211/5*100+F211)/2,0)</f>
@@ -12244,7 +12244,7 @@
         <v>2.42</v>
       </c>
       <c r="F212" s="10" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="H212" s="10">
         <f>ROUND((E212/5*100+F212)/2,0)</f>
@@ -12299,7 +12299,7 @@
         <v>3.46</v>
       </c>
       <c r="F213" s="10" t="n">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="H213" s="10">
         <f>ROUND((E213/5*100+F213)/2,0)</f>
@@ -12354,7 +12354,7 @@
         <v>2.4</v>
       </c>
       <c r="F214" s="10" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="H214" s="10">
         <f>ROUND((E214/5*100+F214)/2,0)</f>
@@ -12409,7 +12409,7 @@
         <v>3.56</v>
       </c>
       <c r="F215" s="10" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H215" s="10">
         <f>ROUND((E215/5*100+F215)/2,0)</f>
@@ -12519,7 +12519,7 @@
         <v>3.62</v>
       </c>
       <c r="F217" s="10" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="H217" s="10">
         <f>ROUND((E217/5*100+F217)/2,0)</f>
@@ -12574,7 +12574,7 @@
         <v>3.55</v>
       </c>
       <c r="F218" s="10" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="H218" s="10">
         <f>ROUND((E218/5*100+F218)/2,0)</f>
@@ -12629,7 +12629,7 @@
         <v>3.39</v>
       </c>
       <c r="F219" s="10" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="H219" s="10">
         <f>ROUND((E219/5*100+F219)/2,0)</f>

</xml_diff>

<commit_message>
Cards: fill estimated budget/box office for 15 new pre-1990 + unreleased films
Filled the empty Budget / World Wide Box Office cells in Movie_DB.xlsx
(all flagged estimated=y) with best estimates, mirrored the same values
into cards.json, and reran build_cards.py to recompute
profit_cost_ratio_pct. Affected: card_221, 224, 236, 239, 240, 246, 247,
250, 260, 262, 263, 264, 265, 275, 303.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -12790,6 +12790,9 @@
       <c r="D222" s="10" t="n">
         <v>2026</v>
       </c>
+      <c r="I222" t="n">
+        <v>1200000000</v>
+      </c>
       <c r="J222" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -12936,6 +12939,9 @@
           <t>y</t>
         </is>
       </c>
+      <c r="K225" t="n">
+        <v>2300000</v>
+      </c>
       <c r="L225" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -13501,10 +13507,16 @@
       <c r="E237" s="10" t="n">
         <v>2.99</v>
       </c>
+      <c r="I237" t="n">
+        <v>3000000</v>
+      </c>
       <c r="J237" s="10" t="inlineStr">
         <is>
           <t>y</t>
         </is>
+      </c>
+      <c r="K237" t="n">
+        <v>1200000</v>
       </c>
       <c r="L237" s="10" t="inlineStr">
         <is>
@@ -13639,10 +13651,16 @@
       <c r="E240" s="10" t="n">
         <v>4.58</v>
       </c>
+      <c r="I240" t="n">
+        <v>4000000</v>
+      </c>
       <c r="J240" s="10" t="inlineStr">
         <is>
           <t>y</t>
         </is>
+      </c>
+      <c r="K240" t="n">
+        <v>2000000</v>
       </c>
       <c r="L240" s="10" t="inlineStr">
         <is>
@@ -13681,10 +13699,16 @@
       <c r="E241" s="10" t="n">
         <v>3.64</v>
       </c>
+      <c r="I241" t="n">
+        <v>6000000</v>
+      </c>
       <c r="J241" s="10" t="inlineStr">
         <is>
           <t>y</t>
         </is>
+      </c>
+      <c r="K241" t="n">
+        <v>2000000</v>
       </c>
       <c r="L241" s="10" t="inlineStr">
         <is>
@@ -13971,6 +13995,9 @@
           <t>y</t>
         </is>
       </c>
+      <c r="K247" t="n">
+        <v>9000000</v>
+      </c>
       <c r="L247" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -14008,10 +14035,16 @@
       <c r="E248" s="10" t="n">
         <v>2.9</v>
       </c>
+      <c r="I248" t="n">
+        <v>4000000</v>
+      </c>
       <c r="J248" s="10" t="inlineStr">
         <is>
           <t>y</t>
         </is>
+      </c>
+      <c r="K248" t="n">
+        <v>2000000</v>
       </c>
       <c r="L248" s="10" t="inlineStr">
         <is>
@@ -14146,6 +14179,9 @@
       <c r="E251" s="10" t="n">
         <v>3.05</v>
       </c>
+      <c r="I251" t="n">
+        <v>2500000</v>
+      </c>
       <c r="J251" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -14623,10 +14659,16 @@
       <c r="E261" s="10" t="n">
         <v>3.81</v>
       </c>
+      <c r="I261" t="n">
+        <v>3000000</v>
+      </c>
       <c r="J261" s="10" t="inlineStr">
         <is>
           <t>y</t>
         </is>
+      </c>
+      <c r="K261" t="n">
+        <v>2000000</v>
       </c>
       <c r="L261" s="10" t="inlineStr">
         <is>
@@ -14713,10 +14755,16 @@
       <c r="E263" s="10" t="n">
         <v>4.4</v>
       </c>
+      <c r="I263" t="n">
+        <v>12000000</v>
+      </c>
       <c r="J263" s="10" t="inlineStr">
         <is>
           <t>y</t>
         </is>
+      </c>
+      <c r="K263" t="n">
+        <v>9000000</v>
       </c>
       <c r="L263" s="10" t="inlineStr">
         <is>
@@ -14755,6 +14803,9 @@
       <c r="E264" s="10" t="n">
         <v>3.94</v>
       </c>
+      <c r="I264" t="n">
+        <v>4000000</v>
+      </c>
       <c r="J264" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -14800,6 +14851,9 @@
       <c r="E265" s="10" t="n">
         <v>3.93</v>
       </c>
+      <c r="I265" t="n">
+        <v>3000000</v>
+      </c>
       <c r="J265" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -14845,6 +14899,9 @@
       <c r="E266" s="10" t="n">
         <v>3.86</v>
       </c>
+      <c r="I266" t="n">
+        <v>5000000</v>
+      </c>
       <c r="J266" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -15330,6 +15387,9 @@
           <t>y</t>
         </is>
       </c>
+      <c r="K276" t="n">
+        <v>45000000</v>
+      </c>
       <c r="L276" s="10" t="inlineStr">
         <is>
           <t>y</t>
@@ -16662,6 +16722,9 @@
       </c>
       <c r="E304" s="10" t="n">
         <v>4.1</v>
+      </c>
+      <c r="I304" t="n">
+        <v>1500000</v>
       </c>
       <c r="J304" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cards: fill card_221 (Spider-Man: Brand New Day) real ratings + runtime
Now released: Letterboxd 4.0, Metacritic user 7.9, runtime 145 min.
audience_score -> 80. Box office still an estimate. cards.json now has
no null values.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -12790,7 +12790,13 @@
       <c r="D222" s="10" t="n">
         <v>2026</v>
       </c>
-      <c r="I222" t="n">
+      <c r="E222" t="n">
+        <v>4</v>
+      </c>
+      <c r="F222" t="n">
+        <v>79</v>
+      </c>
+      <c r="I222" s="10" t="n">
         <v>1200000000</v>
       </c>
       <c r="J222" s="10" t="inlineStr">
@@ -12806,6 +12812,9 @@
           <t>y</t>
         </is>
       </c>
+      <c r="M222" t="n">
+        <v>145</v>
+      </c>
       <c r="N222" s="10" t="n">
         <v>0</v>
       </c>
@@ -12939,7 +12948,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K225" t="n">
+      <c r="K225" s="10" t="n">
         <v>2300000</v>
       </c>
       <c r="L225" s="10" t="inlineStr">
@@ -13507,7 +13516,7 @@
       <c r="E237" s="10" t="n">
         <v>2.99</v>
       </c>
-      <c r="I237" t="n">
+      <c r="I237" s="10" t="n">
         <v>3000000</v>
       </c>
       <c r="J237" s="10" t="inlineStr">
@@ -13515,7 +13524,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K237" t="n">
+      <c r="K237" s="10" t="n">
         <v>1200000</v>
       </c>
       <c r="L237" s="10" t="inlineStr">
@@ -13651,7 +13660,7 @@
       <c r="E240" s="10" t="n">
         <v>4.58</v>
       </c>
-      <c r="I240" t="n">
+      <c r="I240" s="10" t="n">
         <v>4000000</v>
       </c>
       <c r="J240" s="10" t="inlineStr">
@@ -13659,7 +13668,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K240" t="n">
+      <c r="K240" s="10" t="n">
         <v>2000000</v>
       </c>
       <c r="L240" s="10" t="inlineStr">
@@ -13699,7 +13708,7 @@
       <c r="E241" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="I241" t="n">
+      <c r="I241" s="10" t="n">
         <v>6000000</v>
       </c>
       <c r="J241" s="10" t="inlineStr">
@@ -13707,7 +13716,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K241" t="n">
+      <c r="K241" s="10" t="n">
         <v>2000000</v>
       </c>
       <c r="L241" s="10" t="inlineStr">
@@ -13995,7 +14004,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K247" t="n">
+      <c r="K247" s="10" t="n">
         <v>9000000</v>
       </c>
       <c r="L247" s="10" t="inlineStr">
@@ -14035,7 +14044,7 @@
       <c r="E248" s="10" t="n">
         <v>2.9</v>
       </c>
-      <c r="I248" t="n">
+      <c r="I248" s="10" t="n">
         <v>4000000</v>
       </c>
       <c r="J248" s="10" t="inlineStr">
@@ -14043,7 +14052,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K248" t="n">
+      <c r="K248" s="10" t="n">
         <v>2000000</v>
       </c>
       <c r="L248" s="10" t="inlineStr">
@@ -14179,7 +14188,7 @@
       <c r="E251" s="10" t="n">
         <v>3.05</v>
       </c>
-      <c r="I251" t="n">
+      <c r="I251" s="10" t="n">
         <v>2500000</v>
       </c>
       <c r="J251" s="10" t="inlineStr">
@@ -14659,7 +14668,7 @@
       <c r="E261" s="10" t="n">
         <v>3.81</v>
       </c>
-      <c r="I261" t="n">
+      <c r="I261" s="10" t="n">
         <v>3000000</v>
       </c>
       <c r="J261" s="10" t="inlineStr">
@@ -14667,7 +14676,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K261" t="n">
+      <c r="K261" s="10" t="n">
         <v>2000000</v>
       </c>
       <c r="L261" s="10" t="inlineStr">
@@ -14755,7 +14764,7 @@
       <c r="E263" s="10" t="n">
         <v>4.4</v>
       </c>
-      <c r="I263" t="n">
+      <c r="I263" s="10" t="n">
         <v>12000000</v>
       </c>
       <c r="J263" s="10" t="inlineStr">
@@ -14763,7 +14772,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K263" t="n">
+      <c r="K263" s="10" t="n">
         <v>9000000</v>
       </c>
       <c r="L263" s="10" t="inlineStr">
@@ -14803,7 +14812,7 @@
       <c r="E264" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="I264" t="n">
+      <c r="I264" s="10" t="n">
         <v>4000000</v>
       </c>
       <c r="J264" s="10" t="inlineStr">
@@ -14851,7 +14860,7 @@
       <c r="E265" s="10" t="n">
         <v>3.93</v>
       </c>
-      <c r="I265" t="n">
+      <c r="I265" s="10" t="n">
         <v>3000000</v>
       </c>
       <c r="J265" s="10" t="inlineStr">
@@ -14899,7 +14908,7 @@
       <c r="E266" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="I266" t="n">
+      <c r="I266" s="10" t="n">
         <v>5000000</v>
       </c>
       <c r="J266" s="10" t="inlineStr">
@@ -15387,7 +15396,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="K276" t="n">
+      <c r="K276" s="10" t="n">
         <v>45000000</v>
       </c>
       <c r="L276" s="10" t="inlineStr">
@@ -16723,7 +16732,7 @@
       <c r="E304" s="10" t="n">
         <v>4.1</v>
       </c>
-      <c r="I304" t="n">
+      <c r="I304" s="10" t="n">
         <v>1500000</v>
       </c>
       <c r="J304" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Cards: add scraped Metacritic user scores for 48 newer films
Went through all 87 post-card_221 films missing a Metacritic User Rating and
scraped the real user score from metacritic.com where one exists (0-10 ->
stored x10). 48 filled; audience_score recomputed by build_cards.py to blend
Letterboxd + Metacritic instead of the Letterboxd-only fallback.

The remaining 39 films genuinely have no Metacritic user score (mostly
pre-1968 sword-and-sandal / biblical epics that Metacritic never catalogued);
they keep the Letterboxd-only audience_score. Note: metacritic.com/movie/
the-ten-commandments is the 2007 animated film, not the 1956 epic, so
card_234 stays blank.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -12790,10 +12790,10 @@
       <c r="D222" s="10" t="n">
         <v>2026</v>
       </c>
-      <c r="E222" t="n">
+      <c r="E222" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F222" t="n">
+      <c r="F222" s="10" t="n">
         <v>79</v>
       </c>
       <c r="I222" s="10" t="n">
@@ -12812,7 +12812,7 @@
           <t>y</t>
         </is>
       </c>
-      <c r="M222" t="n">
+      <c r="M222" s="10" t="n">
         <v>145</v>
       </c>
       <c r="N222" s="10" t="n">
@@ -12844,6 +12844,9 @@
       <c r="E223" s="10" t="n">
         <v>3.45</v>
       </c>
+      <c r="F223" t="n">
+        <v>68</v>
+      </c>
       <c r="I223" s="10" t="n">
         <v>21000000</v>
       </c>
@@ -13564,6 +13567,9 @@
       <c r="E238" s="10" t="n">
         <v>4.12</v>
       </c>
+      <c r="F238" t="n">
+        <v>87</v>
+      </c>
       <c r="I238" s="10" t="n">
         <v>146900000</v>
       </c>
@@ -13756,6 +13762,9 @@
       <c r="E242" s="10" t="n">
         <v>3.88</v>
       </c>
+      <c r="F242" t="n">
+        <v>79</v>
+      </c>
       <c r="I242" s="10" t="n">
         <v>60000000</v>
       </c>
@@ -13804,6 +13813,9 @@
       <c r="E243" s="10" t="n">
         <v>3.24</v>
       </c>
+      <c r="F243" t="n">
+        <v>73</v>
+      </c>
       <c r="I243" s="10" t="n">
         <v>20000000</v>
       </c>
@@ -13948,6 +13960,9 @@
       <c r="E246" s="10" t="n">
         <v>3.56</v>
       </c>
+      <c r="F246" t="n">
+        <v>75</v>
+      </c>
       <c r="I246" s="10" t="n">
         <v>26600000</v>
       </c>
@@ -14092,6 +14107,9 @@
       <c r="E249" s="10" t="n">
         <v>3.82</v>
       </c>
+      <c r="F249" t="n">
+        <v>75</v>
+      </c>
       <c r="I249" s="10" t="n">
         <v>50100000</v>
       </c>
@@ -14140,6 +14158,9 @@
       <c r="E250" s="10" t="n">
         <v>3.49</v>
       </c>
+      <c r="F250" t="n">
+        <v>67</v>
+      </c>
       <c r="I250" s="10" t="n">
         <v>50000000</v>
       </c>
@@ -14284,6 +14305,9 @@
       <c r="E253" s="10" t="n">
         <v>3.58</v>
       </c>
+      <c r="F253" t="n">
+        <v>66</v>
+      </c>
       <c r="I253" s="10" t="n">
         <v>57800000</v>
       </c>
@@ -14524,6 +14548,9 @@
       <c r="E258" s="10" t="n">
         <v>3.99</v>
       </c>
+      <c r="F258" t="n">
+        <v>79</v>
+      </c>
       <c r="I258" s="10" t="n">
         <v>111700000</v>
       </c>
@@ -14908,6 +14935,9 @@
       <c r="E266" s="10" t="n">
         <v>3.86</v>
       </c>
+      <c r="F266" t="n">
+        <v>78</v>
+      </c>
       <c r="I266" s="10" t="n">
         <v>5000000</v>
       </c>
@@ -15004,6 +15034,9 @@
       <c r="E268" s="10" t="n">
         <v>3.73</v>
       </c>
+      <c r="F268" t="n">
+        <v>72</v>
+      </c>
       <c r="I268" s="10" t="n">
         <v>50700000</v>
       </c>
@@ -15052,6 +15085,9 @@
       <c r="E269" s="10" t="n">
         <v>3.78</v>
       </c>
+      <c r="F269" t="n">
+        <v>68</v>
+      </c>
       <c r="I269" s="10" t="n">
         <v>3500000</v>
       </c>
@@ -15100,6 +15136,9 @@
       <c r="E270" s="10" t="n">
         <v>3.75</v>
       </c>
+      <c r="F270" t="n">
+        <v>75</v>
+      </c>
       <c r="I270" s="10" t="n">
         <v>46800000</v>
       </c>
@@ -15148,6 +15187,9 @@
       <c r="E271" s="10" t="n">
         <v>3.93</v>
       </c>
+      <c r="F271" t="n">
+        <v>77</v>
+      </c>
       <c r="I271" s="10" t="n">
         <v>40400000</v>
       </c>
@@ -15196,6 +15238,9 @@
       <c r="E272" s="10" t="n">
         <v>3.75</v>
       </c>
+      <c r="F272" t="n">
+        <v>81</v>
+      </c>
       <c r="I272" s="10" t="n">
         <v>127800000</v>
       </c>
@@ -15244,6 +15289,9 @@
       <c r="E273" s="10" t="n">
         <v>2.85</v>
       </c>
+      <c r="F273" t="n">
+        <v>63</v>
+      </c>
       <c r="I273" s="10" t="n">
         <v>30900000</v>
       </c>
@@ -15340,6 +15388,9 @@
       <c r="E275" s="10" t="n">
         <v>3.94</v>
       </c>
+      <c r="F275" t="n">
+        <v>81</v>
+      </c>
       <c r="I275" s="10" t="n">
         <v>44000000</v>
       </c>
@@ -15436,6 +15487,9 @@
       <c r="E277" s="10" t="n">
         <v>3.94</v>
       </c>
+      <c r="F277" t="n">
+        <v>81</v>
+      </c>
       <c r="I277" s="10" t="n">
         <v>424200000</v>
       </c>
@@ -15484,6 +15538,9 @@
       <c r="E278" s="10" t="n">
         <v>2.88</v>
       </c>
+      <c r="F278" t="n">
+        <v>57</v>
+      </c>
       <c r="I278" s="10" t="n">
         <v>59000000</v>
       </c>
@@ -15532,6 +15589,9 @@
       <c r="E279" s="10" t="n">
         <v>3.69</v>
       </c>
+      <c r="F279" t="n">
+        <v>78</v>
+      </c>
       <c r="I279" s="10" t="n">
         <v>143000000</v>
       </c>
@@ -15628,6 +15688,9 @@
       <c r="E281" s="10" t="n">
         <v>3.93</v>
       </c>
+      <c r="F281" t="n">
+        <v>81</v>
+      </c>
       <c r="I281" s="10" t="n">
         <v>209000000</v>
       </c>
@@ -15676,6 +15739,9 @@
       <c r="E282" s="10" t="n">
         <v>3.84</v>
       </c>
+      <c r="F282" t="n">
+        <v>83</v>
+      </c>
       <c r="I282" s="10" t="n">
         <v>2264000000</v>
       </c>
@@ -15772,6 +15838,9 @@
       <c r="E284" s="10" t="n">
         <v>3.21</v>
       </c>
+      <c r="F284" t="n">
+        <v>64</v>
+      </c>
       <c r="I284" s="10" t="n">
         <v>67000000</v>
       </c>
@@ -15820,6 +15889,9 @@
       <c r="E285" s="10" t="n">
         <v>3.45</v>
       </c>
+      <c r="F285" t="n">
+        <v>72</v>
+      </c>
       <c r="I285" s="10" t="n">
         <v>215000000</v>
       </c>
@@ -15868,6 +15940,9 @@
       <c r="E286" s="10" t="n">
         <v>3.73</v>
       </c>
+      <c r="F286" t="n">
+        <v>76</v>
+      </c>
       <c r="I286" s="10" t="n">
         <v>193800000</v>
       </c>
@@ -15916,6 +15991,9 @@
       <c r="E287" s="10" t="n">
         <v>3.8</v>
       </c>
+      <c r="F287" t="n">
+        <v>82</v>
+      </c>
       <c r="I287" s="10" t="n">
         <v>456800000</v>
       </c>
@@ -15964,6 +16042,9 @@
       <c r="E288" s="10" t="n">
         <v>2.68</v>
       </c>
+      <c r="F288" t="n">
+        <v>62</v>
+      </c>
       <c r="I288" s="10" t="n">
         <v>12800000</v>
       </c>
@@ -16012,6 +16093,9 @@
       <c r="E289" s="10" t="n">
         <v>3.51</v>
       </c>
+      <c r="F289" t="n">
+        <v>77</v>
+      </c>
       <c r="I289" s="10" t="n">
         <v>497400000</v>
       </c>
@@ -16060,6 +16144,9 @@
       <c r="E290" s="10" t="n">
         <v>2.82</v>
       </c>
+      <c r="F290" t="n">
+        <v>57</v>
+      </c>
       <c r="I290" s="10" t="n">
         <v>167300000</v>
       </c>
@@ -16108,6 +16195,9 @@
       <c r="E291" s="10" t="n">
         <v>3.74</v>
       </c>
+      <c r="F291" t="n">
+        <v>76</v>
+      </c>
       <c r="I291" s="10" t="n">
         <v>218100000</v>
       </c>
@@ -16156,6 +16246,9 @@
       <c r="E292" s="10" t="n">
         <v>2.94</v>
       </c>
+      <c r="F292" t="n">
+        <v>64</v>
+      </c>
       <c r="I292" s="10" t="n">
         <v>211800000</v>
       </c>
@@ -16204,6 +16297,9 @@
       <c r="E293" s="10" t="n">
         <v>2.1</v>
       </c>
+      <c r="F293" t="n">
+        <v>43</v>
+      </c>
       <c r="I293" s="10" t="n">
         <v>269800000</v>
       </c>
@@ -16252,6 +16348,9 @@
       <c r="E294" s="10" t="n">
         <v>3.39</v>
       </c>
+      <c r="F294" t="n">
+        <v>72</v>
+      </c>
       <c r="I294" s="10" t="n">
         <v>39000000</v>
       </c>
@@ -16300,6 +16399,9 @@
       <c r="E295" s="10" t="n">
         <v>3.59</v>
       </c>
+      <c r="F295" t="n">
+        <v>74</v>
+      </c>
       <c r="I295" s="10" t="n">
         <v>275300000</v>
       </c>
@@ -16348,6 +16450,9 @@
       <c r="E296" s="10" t="n">
         <v>2.53</v>
       </c>
+      <c r="F296" t="n">
+        <v>49</v>
+      </c>
       <c r="I296" s="10" t="n">
         <v>268200000</v>
       </c>
@@ -16396,6 +16501,9 @@
       <c r="E297" s="10" t="n">
         <v>2.4</v>
       </c>
+      <c r="F297" t="n">
+        <v>50</v>
+      </c>
       <c r="I297" s="10" t="n">
         <v>117800000</v>
       </c>
@@ -16444,6 +16552,9 @@
       <c r="E298" s="10" t="n">
         <v>2.6</v>
       </c>
+      <c r="F298" t="n">
+        <v>54</v>
+      </c>
       <c r="I298" s="10" t="n">
         <v>359000000</v>
       </c>
@@ -16492,6 +16603,9 @@
       <c r="E299" s="10" t="n">
         <v>3.49</v>
       </c>
+      <c r="F299" t="n">
+        <v>64</v>
+      </c>
       <c r="I299" s="10" t="n">
         <v>9100000</v>
       </c>
@@ -16540,6 +16654,9 @@
       <c r="E300" s="10" t="n">
         <v>4.02</v>
       </c>
+      <c r="F300" t="n">
+        <v>76</v>
+      </c>
       <c r="I300" s="10" t="n">
         <v>24000000</v>
       </c>
@@ -16588,6 +16705,9 @@
       <c r="E301" s="10" t="n">
         <v>3.92</v>
       </c>
+      <c r="F301" t="n">
+        <v>80</v>
+      </c>
       <c r="I301" s="10" t="n">
         <v>8000000</v>
       </c>
@@ -16636,6 +16756,9 @@
       <c r="E302" s="10" t="n">
         <v>3.75</v>
       </c>
+      <c r="F302" t="n">
+        <v>73</v>
+      </c>
       <c r="I302" s="10" t="n">
         <v>30600000</v>
       </c>
@@ -16684,6 +16807,9 @@
       <c r="E303" s="10" t="n">
         <v>3.89</v>
       </c>
+      <c r="F303" t="n">
+        <v>79</v>
+      </c>
       <c r="I303" s="10" t="n">
         <v>411000000</v>
       </c>
@@ -16732,6 +16858,9 @@
       <c r="E304" s="10" t="n">
         <v>4.1</v>
       </c>
+      <c r="F304" t="n">
+        <v>83</v>
+      </c>
       <c r="I304" s="10" t="n">
         <v>1500000</v>
       </c>
@@ -16780,6 +16909,9 @@
       <c r="E305" s="10" t="n">
         <v>4.16</v>
       </c>
+      <c r="F305" t="n">
+        <v>84</v>
+      </c>
       <c r="I305" s="10" t="n">
         <v>983100000</v>
       </c>
@@ -16828,6 +16960,9 @@
       <c r="E306" s="10" t="n">
         <v>2.9</v>
       </c>
+      <c r="F306" t="n">
+        <v>51</v>
+      </c>
       <c r="I306" s="10" t="n">
         <v>222400000</v>
       </c>
@@ -16876,6 +17011,9 @@
       <c r="E307" s="10" t="n">
         <v>4.02</v>
       </c>
+      <c r="F307" t="n">
+        <v>76</v>
+      </c>
       <c r="I307" s="10" t="n">
         <v>158800000</v>
       </c>
@@ -16924,6 +17062,9 @@
       <c r="E308" s="10" t="n">
         <v>4.38</v>
       </c>
+      <c r="F308" t="n">
+        <v>83</v>
+      </c>
       <c r="I308" s="10" t="n">
         <v>714444358</v>
       </c>
@@ -16971,6 +17112,9 @@
       </c>
       <c r="E309" s="10" t="n">
         <v>3.25</v>
+      </c>
+      <c r="F309" t="n">
+        <v>53</v>
       </c>
       <c r="I309" s="10" t="n">
         <v>462700000</v>

</xml_diff>

<commit_message>
Cards: flag direct-to-streaming films, exclude from pool; fix Dogville / Ottoman Lt box office
- New xlsx column "Streaming Release"; build_cards.py reads it into
  streaming_release (bool) and nulls box_office_usd for those titles (their
  theatrical gross is a token awards run or nothing, so profit_cost_ratio_pct
  also goes null).
- CardLoader.load_cards() drops streaming_release cards from the playable pool
  by default; pass include_streaming=true for data tooling. Test count 308->306.
- Flagged: card_300 The Irishman (Netflix 2019), card_303 All Quiet on the
  Western Front (Netflix 2022). These were the only two direct-to-streaming
  titles in the set.
- Data fixes surfaced while re-checking the negative-profit tail:
  card_123 Dogville box office 1.6M -> 16.7M (was US-domestic, not worldwide;
  profit -84% -> +67%); card_020 The Ottoman Lieutenant 1.5M -> 414K (actual
  worldwide gross; -96% -> -99%).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O309"/>
+  <dimension ref="A1:P309"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -489,6 +489,11 @@
           <t>Director Oscar Wins</t>
         </is>
       </c>
+      <c r="P1" s="10" t="inlineStr">
+        <is>
+          <t>Streaming Release</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
@@ -1585,7 +1590,7 @@
         <v/>
       </c>
       <c r="I21" s="19" t="n">
-        <v>1500000</v>
+        <v>414000</v>
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
@@ -7353,7 +7358,7 @@
         <v/>
       </c>
       <c r="I124" s="19" t="n">
-        <v>1600000</v>
+        <v>16700000</v>
       </c>
       <c r="J124" s="12" t="inlineStr">
         <is>
@@ -12844,7 +12849,7 @@
       <c r="E223" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F223" t="n">
+      <c r="F223" s="10" t="n">
         <v>68</v>
       </c>
       <c r="I223" s="10" t="n">
@@ -13567,7 +13572,7 @@
       <c r="E238" s="10" t="n">
         <v>4.12</v>
       </c>
-      <c r="F238" t="n">
+      <c r="F238" s="10" t="n">
         <v>87</v>
       </c>
       <c r="I238" s="10" t="n">
@@ -13762,7 +13767,7 @@
       <c r="E242" s="10" t="n">
         <v>3.88</v>
       </c>
-      <c r="F242" t="n">
+      <c r="F242" s="10" t="n">
         <v>79</v>
       </c>
       <c r="I242" s="10" t="n">
@@ -13813,7 +13818,7 @@
       <c r="E243" s="10" t="n">
         <v>3.24</v>
       </c>
-      <c r="F243" t="n">
+      <c r="F243" s="10" t="n">
         <v>73</v>
       </c>
       <c r="I243" s="10" t="n">
@@ -13960,7 +13965,7 @@
       <c r="E246" s="10" t="n">
         <v>3.56</v>
       </c>
-      <c r="F246" t="n">
+      <c r="F246" s="10" t="n">
         <v>75</v>
       </c>
       <c r="I246" s="10" t="n">
@@ -14107,7 +14112,7 @@
       <c r="E249" s="10" t="n">
         <v>3.82</v>
       </c>
-      <c r="F249" t="n">
+      <c r="F249" s="10" t="n">
         <v>75</v>
       </c>
       <c r="I249" s="10" t="n">
@@ -14158,7 +14163,7 @@
       <c r="E250" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="F250" t="n">
+      <c r="F250" s="10" t="n">
         <v>67</v>
       </c>
       <c r="I250" s="10" t="n">
@@ -14305,7 +14310,7 @@
       <c r="E253" s="10" t="n">
         <v>3.58</v>
       </c>
-      <c r="F253" t="n">
+      <c r="F253" s="10" t="n">
         <v>66</v>
       </c>
       <c r="I253" s="10" t="n">
@@ -14548,7 +14553,7 @@
       <c r="E258" s="10" t="n">
         <v>3.99</v>
       </c>
-      <c r="F258" t="n">
+      <c r="F258" s="10" t="n">
         <v>79</v>
       </c>
       <c r="I258" s="10" t="n">
@@ -14935,7 +14940,7 @@
       <c r="E266" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="F266" t="n">
+      <c r="F266" s="10" t="n">
         <v>78</v>
       </c>
       <c r="I266" s="10" t="n">
@@ -15034,7 +15039,7 @@
       <c r="E268" s="10" t="n">
         <v>3.73</v>
       </c>
-      <c r="F268" t="n">
+      <c r="F268" s="10" t="n">
         <v>72</v>
       </c>
       <c r="I268" s="10" t="n">
@@ -15085,7 +15090,7 @@
       <c r="E269" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F269" t="n">
+      <c r="F269" s="10" t="n">
         <v>68</v>
       </c>
       <c r="I269" s="10" t="n">
@@ -15136,7 +15141,7 @@
       <c r="E270" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F270" t="n">
+      <c r="F270" s="10" t="n">
         <v>75</v>
       </c>
       <c r="I270" s="10" t="n">
@@ -15187,7 +15192,7 @@
       <c r="E271" s="10" t="n">
         <v>3.93</v>
       </c>
-      <c r="F271" t="n">
+      <c r="F271" s="10" t="n">
         <v>77</v>
       </c>
       <c r="I271" s="10" t="n">
@@ -15238,7 +15243,7 @@
       <c r="E272" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F272" t="n">
+      <c r="F272" s="10" t="n">
         <v>81</v>
       </c>
       <c r="I272" s="10" t="n">
@@ -15289,7 +15294,7 @@
       <c r="E273" s="10" t="n">
         <v>2.85</v>
       </c>
-      <c r="F273" t="n">
+      <c r="F273" s="10" t="n">
         <v>63</v>
       </c>
       <c r="I273" s="10" t="n">
@@ -15388,7 +15393,7 @@
       <c r="E275" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="F275" t="n">
+      <c r="F275" s="10" t="n">
         <v>81</v>
       </c>
       <c r="I275" s="10" t="n">
@@ -15487,7 +15492,7 @@
       <c r="E277" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="F277" t="n">
+      <c r="F277" s="10" t="n">
         <v>81</v>
       </c>
       <c r="I277" s="10" t="n">
@@ -15538,7 +15543,7 @@
       <c r="E278" s="10" t="n">
         <v>2.88</v>
       </c>
-      <c r="F278" t="n">
+      <c r="F278" s="10" t="n">
         <v>57</v>
       </c>
       <c r="I278" s="10" t="n">
@@ -15589,7 +15594,7 @@
       <c r="E279" s="10" t="n">
         <v>3.69</v>
       </c>
-      <c r="F279" t="n">
+      <c r="F279" s="10" t="n">
         <v>78</v>
       </c>
       <c r="I279" s="10" t="n">
@@ -15688,7 +15693,7 @@
       <c r="E281" s="10" t="n">
         <v>3.93</v>
       </c>
-      <c r="F281" t="n">
+      <c r="F281" s="10" t="n">
         <v>81</v>
       </c>
       <c r="I281" s="10" t="n">
@@ -15739,7 +15744,7 @@
       <c r="E282" s="10" t="n">
         <v>3.84</v>
       </c>
-      <c r="F282" t="n">
+      <c r="F282" s="10" t="n">
         <v>83</v>
       </c>
       <c r="I282" s="10" t="n">
@@ -15838,7 +15843,7 @@
       <c r="E284" s="10" t="n">
         <v>3.21</v>
       </c>
-      <c r="F284" t="n">
+      <c r="F284" s="10" t="n">
         <v>64</v>
       </c>
       <c r="I284" s="10" t="n">
@@ -15889,7 +15894,7 @@
       <c r="E285" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F285" t="n">
+      <c r="F285" s="10" t="n">
         <v>72</v>
       </c>
       <c r="I285" s="10" t="n">
@@ -15940,7 +15945,7 @@
       <c r="E286" s="10" t="n">
         <v>3.73</v>
       </c>
-      <c r="F286" t="n">
+      <c r="F286" s="10" t="n">
         <v>76</v>
       </c>
       <c r="I286" s="10" t="n">
@@ -15991,7 +15996,7 @@
       <c r="E287" s="10" t="n">
         <v>3.8</v>
       </c>
-      <c r="F287" t="n">
+      <c r="F287" s="10" t="n">
         <v>82</v>
       </c>
       <c r="I287" s="10" t="n">
@@ -16042,7 +16047,7 @@
       <c r="E288" s="10" t="n">
         <v>2.68</v>
       </c>
-      <c r="F288" t="n">
+      <c r="F288" s="10" t="n">
         <v>62</v>
       </c>
       <c r="I288" s="10" t="n">
@@ -16093,7 +16098,7 @@
       <c r="E289" s="10" t="n">
         <v>3.51</v>
       </c>
-      <c r="F289" t="n">
+      <c r="F289" s="10" t="n">
         <v>77</v>
       </c>
       <c r="I289" s="10" t="n">
@@ -16144,7 +16149,7 @@
       <c r="E290" s="10" t="n">
         <v>2.82</v>
       </c>
-      <c r="F290" t="n">
+      <c r="F290" s="10" t="n">
         <v>57</v>
       </c>
       <c r="I290" s="10" t="n">
@@ -16195,7 +16200,7 @@
       <c r="E291" s="10" t="n">
         <v>3.74</v>
       </c>
-      <c r="F291" t="n">
+      <c r="F291" s="10" t="n">
         <v>76</v>
       </c>
       <c r="I291" s="10" t="n">
@@ -16246,7 +16251,7 @@
       <c r="E292" s="10" t="n">
         <v>2.94</v>
       </c>
-      <c r="F292" t="n">
+      <c r="F292" s="10" t="n">
         <v>64</v>
       </c>
       <c r="I292" s="10" t="n">
@@ -16297,7 +16302,7 @@
       <c r="E293" s="10" t="n">
         <v>2.1</v>
       </c>
-      <c r="F293" t="n">
+      <c r="F293" s="10" t="n">
         <v>43</v>
       </c>
       <c r="I293" s="10" t="n">
@@ -16348,7 +16353,7 @@
       <c r="E294" s="10" t="n">
         <v>3.39</v>
       </c>
-      <c r="F294" t="n">
+      <c r="F294" s="10" t="n">
         <v>72</v>
       </c>
       <c r="I294" s="10" t="n">
@@ -16399,7 +16404,7 @@
       <c r="E295" s="10" t="n">
         <v>3.59</v>
       </c>
-      <c r="F295" t="n">
+      <c r="F295" s="10" t="n">
         <v>74</v>
       </c>
       <c r="I295" s="10" t="n">
@@ -16450,7 +16455,7 @@
       <c r="E296" s="10" t="n">
         <v>2.53</v>
       </c>
-      <c r="F296" t="n">
+      <c r="F296" s="10" t="n">
         <v>49</v>
       </c>
       <c r="I296" s="10" t="n">
@@ -16501,7 +16506,7 @@
       <c r="E297" s="10" t="n">
         <v>2.4</v>
       </c>
-      <c r="F297" t="n">
+      <c r="F297" s="10" t="n">
         <v>50</v>
       </c>
       <c r="I297" s="10" t="n">
@@ -16552,7 +16557,7 @@
       <c r="E298" s="10" t="n">
         <v>2.6</v>
       </c>
-      <c r="F298" t="n">
+      <c r="F298" s="10" t="n">
         <v>54</v>
       </c>
       <c r="I298" s="10" t="n">
@@ -16603,7 +16608,7 @@
       <c r="E299" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="F299" t="n">
+      <c r="F299" s="10" t="n">
         <v>64</v>
       </c>
       <c r="I299" s="10" t="n">
@@ -16654,7 +16659,7 @@
       <c r="E300" s="10" t="n">
         <v>4.02</v>
       </c>
-      <c r="F300" t="n">
+      <c r="F300" s="10" t="n">
         <v>76</v>
       </c>
       <c r="I300" s="10" t="n">
@@ -16705,17 +16710,11 @@
       <c r="E301" s="10" t="n">
         <v>3.92</v>
       </c>
-      <c r="F301" t="n">
+      <c r="F301" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I301" s="10" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="J301" s="10" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
+      <c r="I301" s="10" t="n"/>
+      <c r="J301" s="10" t="n"/>
       <c r="K301" s="10" t="n">
         <v>200000000</v>
       </c>
@@ -16733,6 +16732,11 @@
       <c r="O301" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="P301" s="10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="10" t="inlineStr">
@@ -16756,7 +16760,7 @@
       <c r="E302" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F302" t="n">
+      <c r="F302" s="10" t="n">
         <v>73</v>
       </c>
       <c r="I302" s="10" t="n">
@@ -16807,7 +16811,7 @@
       <c r="E303" s="10" t="n">
         <v>3.89</v>
       </c>
-      <c r="F303" t="n">
+      <c r="F303" s="10" t="n">
         <v>79</v>
       </c>
       <c r="I303" s="10" t="n">
@@ -16858,17 +16862,11 @@
       <c r="E304" s="10" t="n">
         <v>4.1</v>
       </c>
-      <c r="F304" t="n">
+      <c r="F304" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I304" s="10" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="J304" s="10" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
+      <c r="I304" s="10" t="n"/>
+      <c r="J304" s="10" t="n"/>
       <c r="K304" s="10" t="n">
         <v>20000000</v>
       </c>
@@ -16886,6 +16884,11 @@
       <c r="O304" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="P304" s="10" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="10" t="inlineStr">
@@ -16909,7 +16912,7 @@
       <c r="E305" s="10" t="n">
         <v>4.16</v>
       </c>
-      <c r="F305" t="n">
+      <c r="F305" s="10" t="n">
         <v>84</v>
       </c>
       <c r="I305" s="10" t="n">
@@ -16960,7 +16963,7 @@
       <c r="E306" s="10" t="n">
         <v>2.9</v>
       </c>
-      <c r="F306" t="n">
+      <c r="F306" s="10" t="n">
         <v>51</v>
       </c>
       <c r="I306" s="10" t="n">
@@ -17011,7 +17014,7 @@
       <c r="E307" s="10" t="n">
         <v>4.02</v>
       </c>
-      <c r="F307" t="n">
+      <c r="F307" s="10" t="n">
         <v>76</v>
       </c>
       <c r="I307" s="10" t="n">
@@ -17062,7 +17065,7 @@
       <c r="E308" s="10" t="n">
         <v>4.38</v>
       </c>
-      <c r="F308" t="n">
+      <c r="F308" s="10" t="n">
         <v>83</v>
       </c>
       <c r="I308" s="10" t="n">
@@ -17113,7 +17116,7 @@
       <c r="E309" s="10" t="n">
         <v>3.25</v>
       </c>
-      <c r="F309" t="n">
+      <c r="F309" s="10" t="n">
         <v>53</v>
       </c>
       <c r="I309" s="10" t="n">

</xml_diff>